<commit_message>
Add columns-withimg-light block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 10
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-news-press-release.report.xlsx
+++ b/tools/importer/reports/import-news-press-release.report.xlsx
@@ -388,7 +388,7 @@
     <t>news/hidden-signs-of-financial-abuse.report.json</t>
   </si>
   <si>
-    <t>["nav-anchor-light","columns-withimg-light","columns"]</t>
+    <t>["nav-anchor-light","columns-withimg-light","columns-withimg-light","columns"]</t>
   </si>
   <si>
     <t>news/hidden-signs-of-financial-abuse</t>
@@ -397,7 +397,7 @@
     <t>news-press-release</t>
   </si>
   <si>
-    <t>2026-09-26T13:15:55.937Z</t>
+    <t>2026-09-26T13:40:35.880Z</t>
   </si>
   <si>
     <t>News - Study finds banking records reveal the hidden signs of financial abuse - University of Nottingham</t>

</xml_diff>